<commit_message>
Version 30 Final Release
</commit_message>
<xml_diff>
--- a/outputs/Block2_2026_Fold_Forecasts_v12.xlsx
+++ b/outputs/Block2_2026_Fold_Forecasts_v12.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
   <si>
     <t>Omitted Historical Cycle</t>
   </si>
@@ -70,7 +70,10 @@
     <t>ExpectedVoteAnchor</t>
   </si>
   <si>
-    <t>Ridge</t>
+    <t>Derived downstream from 435 races</t>
+  </si>
+  <si>
+    <t>Derived downstream from Senate races</t>
   </si>
 </sst>
 </file>
@@ -483,28 +486,28 @@
         <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F2">
-        <v>52.42150155486451</v>
+        <v>52.8453434096466</v>
       </c>
       <c r="G2">
-        <v>44.7784984451355</v>
+        <v>44.35465659035341</v>
       </c>
       <c r="H2">
-        <v>7.643003109729013</v>
+        <v>8.490686819293186</v>
       </c>
       <c r="I2">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="J2">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="K2">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L2">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -521,28 +524,28 @@
         <v>18</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F3">
-        <v>52.42150155486451</v>
+        <v>52.8453434096466</v>
       </c>
       <c r="G3">
-        <v>44.7784984451355</v>
+        <v>44.3546565903534</v>
       </c>
       <c r="H3">
-        <v>7.643003109729007</v>
+        <v>8.490686819293192</v>
       </c>
       <c r="I3">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="J3">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="K3">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="L3">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -559,28 +562,28 @@
         <v>18</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F4">
-        <v>52.40801865837405</v>
+        <v>52.83175150033341</v>
       </c>
       <c r="G4">
-        <v>44.76698134162594</v>
+        <v>44.34324849966659</v>
       </c>
       <c r="H4">
-        <v>7.641037316748111</v>
+        <v>8.488503000666825</v>
       </c>
       <c r="I4">
-        <v>237</v>
+        <v>215</v>
       </c>
       <c r="J4">
-        <v>198</v>
+        <v>220</v>
       </c>
       <c r="K4">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="L4">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -597,28 +600,28 @@
         <v>18</v>
       </c>
       <c r="E5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F5">
-        <v>52.20577521101733</v>
+        <v>52.6278728606357</v>
       </c>
       <c r="G5">
-        <v>44.59422478898268</v>
+        <v>44.17212713936431</v>
       </c>
       <c r="H5">
-        <v>7.611550422034657</v>
+        <v>8.455745721271402</v>
       </c>
       <c r="I5">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="J5">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="K5">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="L5">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -635,28 +638,28 @@
         <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F6">
-        <v>52.32712127943137</v>
+        <v>52.75020004445433</v>
       </c>
       <c r="G6">
-        <v>44.69787872056864</v>
+        <v>44.27479995554567</v>
       </c>
       <c r="H6">
-        <v>7.629242558862726</v>
+        <v>8.475400088908657</v>
       </c>
       <c r="I6">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="J6">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="K6">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="L6">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final Version 15 monitored
</commit_message>
<xml_diff>
--- a/outputs/Block2_2026_Fold_Forecasts_v12.xlsx
+++ b/outputs/Block2_2026_Fold_Forecasts_v12.xlsx
@@ -489,13 +489,13 @@
         <v>19</v>
       </c>
       <c r="F2">
-        <v>53.02206593406594</v>
+        <v>52.86984957488554</v>
       </c>
       <c r="G2">
-        <v>44.17793406593407</v>
+        <v>44.33015042511447</v>
       </c>
       <c r="H2">
-        <v>8.844131868131877</v>
+        <v>8.539699149771074</v>
       </c>
       <c r="I2">
         <v>215</v>
@@ -527,13 +527,13 @@
         <v>19</v>
       </c>
       <c r="F3">
-        <v>53.02206593406594</v>
+        <v>52.86984957488554</v>
       </c>
       <c r="G3">
-        <v>44.17793406593407</v>
+        <v>44.33015042511446</v>
       </c>
       <c r="H3">
-        <v>8.844131868131866</v>
+        <v>8.53969914977108</v>
       </c>
       <c r="I3">
         <v>215</v>
@@ -565,13 +565,13 @@
         <v>19</v>
       </c>
       <c r="F4">
-        <v>53.00842857142858</v>
+        <v>52.85625136254632</v>
       </c>
       <c r="G4">
-        <v>44.16657142857143</v>
+        <v>44.31874863745368</v>
       </c>
       <c r="H4">
-        <v>8.841857142857151</v>
+        <v>8.537502725092633</v>
       </c>
       <c r="I4">
         <v>215</v>
@@ -603,13 +603,13 @@
         <v>19</v>
       </c>
       <c r="F5">
-        <v>52.80386813186814</v>
+        <v>52.65227817745804</v>
       </c>
       <c r="G5">
-        <v>43.99613186813187</v>
+        <v>44.14772182254198</v>
       </c>
       <c r="H5">
-        <v>8.807736263736265</v>
+        <v>8.504556354916055</v>
       </c>
       <c r="I5">
         <v>215</v>
@@ -641,13 +641,13 @@
         <v>19</v>
       </c>
       <c r="F6">
-        <v>52.92660439560441</v>
+        <v>52.77466208851101</v>
       </c>
       <c r="G6">
-        <v>44.09839560439561</v>
+        <v>44.250337911489</v>
       </c>
       <c r="H6">
-        <v>8.828208791208796</v>
+        <v>8.524324177022002</v>
       </c>
       <c r="I6">
         <v>215</v>

</xml_diff>